<commit_message>
Canonize 9x9 source coverage
</commit_message>
<xml_diff>
--- a/NewLogic 03.05.2026/ST_Friction_Point_Lookup_updated.xlsx
+++ b/NewLogic 03.05.2026/ST_Friction_Point_Lookup_updated.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Friction_Lookup" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECS_Matrix" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derivation_Method" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk_Category_Tagging" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v3_1_Build_Notes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Friction_Lookup" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ECS_Matrix" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Derivation_Method" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Risk_Category_Tagging" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="v3_1_Build_Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -6021,7 +6021,7 @@
       </c>
       <c r="K4" s="126" t="inlineStr">
         <is>
-          <t>64.7</t>
+          <t>64.7 →FP</t>
         </is>
       </c>
     </row>
@@ -6074,7 +6074,7 @@
       </c>
       <c r="K5" s="128" t="inlineStr">
         <is>
-          <t>35.3</t>
+          <t>35.3 →FP</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6127,7 @@
       </c>
       <c r="K6" s="126" t="inlineStr">
         <is>
-          <t>64.7</t>
+          <t>64.7 →FP</t>
         </is>
       </c>
     </row>
@@ -6180,7 +6180,7 @@
       </c>
       <c r="K7" s="129" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>73.5 →FP</t>
         </is>
       </c>
     </row>
@@ -6233,7 +6233,7 @@
       </c>
       <c r="K8" s="129" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>70.6 →FP</t>
         </is>
       </c>
     </row>
@@ -6286,7 +6286,7 @@
       </c>
       <c r="K9" s="126" t="inlineStr">
         <is>
-          <t>61.8</t>
+          <t>61.8 →FP</t>
         </is>
       </c>
     </row>
@@ -6339,7 +6339,7 @@
       </c>
       <c r="K10" s="128" t="inlineStr">
         <is>
-          <t>35.3</t>
+          <t>35.3 →FP</t>
         </is>
       </c>
     </row>
@@ -6392,7 +6392,7 @@
       </c>
       <c r="K11" s="129" t="inlineStr">
         <is>
-          <t>91.2</t>
+          <t>91.2 →FP</t>
         </is>
       </c>
     </row>
@@ -6404,42 +6404,42 @@
       </c>
       <c r="C12" s="126" t="inlineStr">
         <is>
-          <t>64.7</t>
+          <t>64.7 →FP</t>
         </is>
       </c>
       <c r="D12" s="128" t="inlineStr">
         <is>
-          <t>35.3</t>
+          <t>35.3 →FP</t>
         </is>
       </c>
       <c r="E12" s="126" t="inlineStr">
         <is>
-          <t>64.7</t>
+          <t>64.7 →FP</t>
         </is>
       </c>
       <c r="F12" s="129" t="inlineStr">
         <is>
-          <t>73.5</t>
+          <t>73.5 →FP</t>
         </is>
       </c>
       <c r="G12" s="129" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>70.6 →FP</t>
         </is>
       </c>
       <c r="H12" s="126" t="inlineStr">
         <is>
-          <t>61.8</t>
+          <t>61.8 →FP</t>
         </is>
       </c>
       <c r="I12" s="128" t="inlineStr">
         <is>
-          <t>35.3</t>
+          <t>35.3 →FP</t>
         </is>
       </c>
       <c r="J12" s="129" t="inlineStr">
         <is>
-          <t>91.2</t>
+          <t>91.2 →FP</t>
         </is>
       </c>
       <c r="K12" s="131" t="inlineStr">
@@ -6470,7 +6470,7 @@
     <row r="15">
       <c r="A15" s="136" t="inlineStr">
         <is>
-          <t>STP/STJ scores canonized June 2026 — derivation: ST_ECS_Derivation_Method_v1.xlsx (ECS = 100 × (1 − C/34), Net Effect conflict method, Reproduction Test 28/28). No →FP marker: STP/STJ friction-point narratives are not yet authored in Friction_Lookup (16 directed rows pending).</t>
+          <t>STP/STJ scores and friction-point narratives canonized June 2026 — derivation: ST_ECS_Derivation_Method_v1.xlsx / ST_ECS_v1_9x9_canonical_source.xlsx. ECS = 100 × (1 − C/34), Net Effect conflict method, Reproduction Test 28/28. All 72 directed pairs now have ECS scores, friction-point narratives, early-warning signals, primary conflicted resources, and risk-category tags.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Retire verdict language from friction watchpoints
</commit_message>
<xml_diff>
--- a/NewLogic 03.05.2026/ST_Friction_Point_Lookup_updated.xlsx
+++ b/NewLogic 03.05.2026/ST_Friction_Point_Lookup_updated.xlsx
@@ -3025,7 +3025,7 @@
       </c>
       <c r="F35" s="83" t="inlineStr">
         <is>
-          <t>Loyalty versus performance authority. NF/SFJ authority belongs to those most closely associated with the founding narrative. NT/STJ authority belongs to those with the strongest measurable results. These are structurally incompatible. NT/STJ's installation of performance-based authority displaces NF/SFJ's narrative-based authority figures, who typically respond by building internal opposition to the integration.</t>
+          <t>Loyalty versus performance authority. NF/SFJ authority belongs to those most closely associated with the founding narrative; NT/STJ authority belongs to those with the strongest measurable results. Watch whether performance-based authority displaces narrative-based authority before trust-preserving routines are understood. If narrative-linked leaders lose decision visibility and informal opposition rises, the friction thesis strengthens. If authority migration is explicit, accepted, and documented, the risk should be downgraded.</t>
         </is>
       </c>
       <c r="G35" s="84" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="H35" s="85" t="inlineStr">
         <is>
-          <t>Within 30 days: observe how NF/SFJ leaders respond when NT/STJ management asks 'what is the evidence for this?' about a core organisational practice. NF/SFJ environments do not recognise evidence as a valid challenge mechanism — the response will be reframing, not engagement. If this pattern appears in the first senior meeting, the structural incompatibility is confirmed.</t>
+          <t>Within 30 days: observe how NF/SFJ leaders respond when NT/STJ management asks "what is the evidence for this?" about a core organisational practice. If the response shifts from evidence review into mission-framing or identity protection, that is a signal the friction thesis is active. If leaders engage the evidence directly and adjust the practice, the incompatibility signal weakens and the target read should be reviewed.</t>
         </is>
       </c>
       <c r="I35" s="86" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="E42" s="82" t="inlineStr">
         <is>
-          <t>Empirical test versus relational authority conflict. SFJ/SFP decisions are made by the most trusted person — trust defined by relationship tenure. NT/STP resolves disagreements through empirical testing. The first major decision where NT/STP proposes a live test and SFJ/SFP resists because the process violates established custom defines the integration trajectory. Both mechanisms are internally coherent; they are structurally incompatible.</t>
+          <t>Empirical test versus relational authority. SFJ/SFP decisions are made by the most trusted person, with trust defined by relationship tenure; NT/STP resolves disagreements through empirical testing. The first major decision where NT/STP proposes a live test and SFJ/SFP resists because the process breaks established custom is the signal to watch. If resistance hardens and the test is blocked on grounds of custom rather than merit, the friction thesis strengthens. If the test proceeds and results are accepted into the decision, the signal weakens. Both mechanisms are internally coherent; the question is which becomes primary after close.</t>
         </is>
       </c>
       <c r="F42" s="83" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="F44" s="83" t="inlineStr">
         <is>
-          <t>Throughput efficiency versus intelligent failure tolerance. SFP/SFJ optimises for throughput — high turnover is a design feature. NT/STP treats not-testing as the primary failure. These are structurally incompatible: NT/STP's tolerance for intelligent failure and its investment in experimental capacity are direct costs to SFP/SFJ's throughput model.</t>
+          <t>Throughput efficiency versus failure tolerance. SFP/SFJ optimises for throughput, treating high turnover as a design feature; NT/STP treats not-testing as the primary failure and invests in experimental capacity. Watch whether NT/STP's experimental investment is absorbed as a throughput cost. If experimental capacity is cut to protect throughput targets, the friction thesis strengthens. If both are explicitly budgeted and reconciled, the risk should be downgraded.</t>
         </is>
       </c>
       <c r="G44" s="84" t="inlineStr">

</xml_diff>

<commit_message>
fix: enforce friction direction integrity
</commit_message>
<xml_diff>
--- a/NewLogic 03.05.2026/ST_Friction_Point_Lookup_updated.xlsx
+++ b/NewLogic 03.05.2026/ST_Friction_Point_Lookup_updated.xlsx
@@ -1699,7 +1699,7 @@
       </c>
       <c r="I10" s="86" t="inlineStr">
         <is>
-          <t>Trust (+NF/NT vs −STJ/STP), Knowledge (+NF/NT vs −STJ/STP), Energy (+NF/NT vs −STJ/STP)</t>
+          <t>Trust (+NF/NT vs −STJ/STP), Knowledge (+NF/NT vs −STJ/STP), Energy (+NF/NT vs +STJ/STP)</t>
         </is>
       </c>
       <c r="J10" s="87" t="inlineStr">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="I22" s="86" t="inlineStr">
         <is>
-          <t>Organisation/System (~NF/SFP vs ~NF/NT), Will/Discipline (~NF/SFP vs +NF/NT)</t>
+          <t>Organisation/System (-NF/SFP vs ~NF/NT), Will/Discipline (~NF/SFP vs +NF/NT)</t>
         </is>
       </c>
       <c r="J22" s="87" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="I31" s="86" t="inlineStr">
         <is>
-          <t>Knowledge (+NF/NT vs +NT/STJ — but different logic: shared vs competitive), Trust (+NF/NT vs ~NT/STJ), Creativity (+NF/NT vs +NT/STJ — but commodified)</t>
+          <t>Knowledge (+NT/STJ vs +NF/NT — but different logic: shared vs competitive), Trust (~NT/STJ vs +NF/NT), Creativity (+NT/STJ vs +NF/NT — but commodified)</t>
         </is>
       </c>
       <c r="J31" s="92" t="inlineStr">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="I39" s="91" t="inlineStr">
         <is>
-          <t>Knowledge (+NF/NT vs +NT/STP — same effect but different logic: truth vs application), Organisation/System (~NF/NT vs ~NT/STP — both low but for different reasons)</t>
+          <t>Knowledge (+NT/STP vs +NF/NT — same effect but different logic: truth vs application), Organisation/System (~NT/STP vs ~NF/NT — both low but for different reasons)</t>
         </is>
       </c>
       <c r="J39" s="92" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="I66" s="91" t="inlineStr">
         <is>
-          <t>Trust (+SFJ/SFP vs −STJ/STP), Health (+SFJ/SFP vs ~STJ/STP), Connections (+SFJ/SFP vs ~STJ/STP)</t>
+          <t>Trust (−STJ/STP vs +SFJ/SFP), Health (~STJ/STP vs +SFJ/SFP), Connections (~STJ/STP vs +SFJ/SFP)</t>
         </is>
       </c>
       <c r="J66" s="87" t="inlineStr">

</xml_diff>